<commit_message>
lagde admitans funksjon i klassen
</commit_message>
<xml_diff>
--- a/Grid/GridVersion1.xlsx
+++ b/Grid/GridVersion1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0348cbc925570652/Eldig sem. 3/IELET2118/Prosjekt/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0348cbc925570652/Master/Kraftsystemer/Kraftsystemer-2/Grid/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="206" documentId="8_{3C642C3D-EC28-4A74-B6EC-7A1541F07EDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C761D306-71B2-4FBD-97C7-4B9150FCD962}"/>
+  <xr:revisionPtr revIDLastSave="211" documentId="8_{3C642C3D-EC28-4A74-B6EC-7A1541F07EDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4501C804-12EF-47C2-AEBE-EEB495381B3E}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="8810" yWindow="1700" windowWidth="10390" windowHeight="5490" xr2:uid="{E6D3FD58-6DB6-4988-B229-9B990EF92238}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{E6D3FD58-6DB6-4988-B229-9B990EF92238}"/>
   </bookViews>
   <sheets>
     <sheet name="BranchData" sheetId="1" r:id="rId1"/>
@@ -255,10 +255,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -563,6 +559,7 @@
   <cols>
     <col min="3" max="3" width="12.26953125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.81640625" customWidth="1"/>
+    <col min="6" max="6" width="28.81640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1047,6 +1044,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="f922d515-0715-47d2-81b1-ef00605e1c6c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005ACA8563C35EAC4DA458C96C86289442" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d60f1ee50480cf6a29d9af1e44ae1b59">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="f922d515-0715-47d2-81b1-ef00605e1c6c" xmlns:ns4="7451329a-7d84-4aff-a31d-bae55e338dcf" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b15a621f4bf9d812834242f4566d6849" ns3:_="" ns4:_="">
     <xsd:import namespace="f922d515-0715-47d2-81b1-ef00605e1c6c"/>
@@ -1241,24 +1255,25 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75012CDF-1A50-4E16-9241-25F524158EA8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f922d515-0715-47d2-81b1-ef00605e1c6c"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="f922d515-0715-47d2-81b1-ef00605e1c6c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A7D9F204-95DA-4997-975F-50AB2C8864E5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B1C0A06D-1972-47EB-AEC3-64052A311886}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1275,22 +1290,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A7D9F204-95DA-4997-975F-50AB2C8864E5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75012CDF-1A50-4E16-9241-25F524158EA8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="f922d515-0715-47d2-81b1-ef00605e1c6c"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>